<commit_message>
add fusemoe w4a8 TP4\2\1 bestconfig
</commit_message>
<xml_diff>
--- a/test/moe_marlin/moe_w4a8/marlin_prof.xlsx
+++ b/test/moe_marlin/moe_w4a8/marlin_prof.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,10 +498,10 @@
         <v>8</v>
       </c>
       <c r="H2" t="n">
-        <v>86.73128822445869</v>
+        <v>72.06015811860561</v>
       </c>
       <c r="I2" t="n">
-        <v>41.10566117614508</v>
+        <v>42.23046508058906</v>
       </c>
     </row>
     <row r="3">
@@ -527,10 +527,10 @@
         <v>8</v>
       </c>
       <c r="H3" t="n">
-        <v>126.4725230634212</v>
+        <v>115.4141440391541</v>
       </c>
       <c r="I3" t="n">
-        <v>68.12477395683527</v>
+        <v>66.37633095681667</v>
       </c>
     </row>
     <row r="4">
@@ -556,10 +556,10 @@
         <v>8</v>
       </c>
       <c r="H4" t="n">
-        <v>206.7767630666494</v>
+        <v>204.4128528833389</v>
       </c>
       <c r="I4" t="n">
-        <v>114.0467420816422</v>
+        <v>117.2862790152431</v>
       </c>
     </row>
     <row r="5">
@@ -585,10 +585,10 @@
         <v>8</v>
       </c>
       <c r="H5" t="n">
-        <v>391.0774291753769</v>
+        <v>358.0316828489304</v>
       </c>
       <c r="I5" t="n">
-        <v>340.0564451664686</v>
+        <v>205.7816171497107</v>
       </c>
     </row>
     <row r="6">
@@ -614,10 +614,10 @@
         <v>8</v>
       </c>
       <c r="H6" t="n">
-        <v>589.9235138893127</v>
+        <v>595.7887712717056</v>
       </c>
       <c r="I6" t="n">
-        <v>340.3504872620106</v>
+        <v>355.5472338199615</v>
       </c>
     </row>
     <row r="7">
@@ -643,10 +643,10 @@
         <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>929.6833935976028</v>
+        <v>940.7008419632912</v>
       </c>
       <c r="I7" t="n">
-        <v>540.3450418710709</v>
+        <v>557.7685605287552</v>
       </c>
     </row>
     <row r="8">
@@ -672,10 +672,10 @@
         <v>8</v>
       </c>
       <c r="H8" t="n">
-        <v>1284.151927947998</v>
+        <v>1299.073054671288</v>
       </c>
       <c r="I8" t="n">
-        <v>745.028977394104</v>
+        <v>767.1804723739624</v>
       </c>
     </row>
     <row r="9">
@@ -701,10 +701,10 @@
         <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>1466.77931022644</v>
+        <v>1495.833188056946</v>
       </c>
       <c r="I9" t="n">
-        <v>867.2939409017563</v>
+        <v>888.6482067704201</v>
       </c>
     </row>
     <row r="10">
@@ -730,10 +730,10 @@
         <v>8</v>
       </c>
       <c r="H10" t="n">
-        <v>1543.015846729279</v>
+        <v>1570.109223723412</v>
       </c>
       <c r="I10" t="n">
-        <v>919.654431283474</v>
+        <v>942.3191874027252</v>
       </c>
     </row>
     <row r="11">
@@ -759,10 +759,184 @@
         <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>1797.291633248329</v>
+        <v>1827.554886341095</v>
       </c>
       <c r="I11" t="n">
-        <v>1033.272795557976</v>
+        <v>1052.949891448021</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E12" t="n">
+        <v>512</v>
+      </c>
+      <c r="F12" t="n">
+        <v>256</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1752.814930319786</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1262.710780620575</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E13" t="n">
+        <v>512</v>
+      </c>
+      <c r="F13" t="n">
+        <v>256</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1719.860273480415</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1900.462051749229</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E14" t="n">
+        <v>512</v>
+      </c>
+      <c r="F14" t="n">
+        <v>256</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2244.859130382538</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2987.312002658844</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6144</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E15" t="n">
+        <v>512</v>
+      </c>
+      <c r="F15" t="n">
+        <v>256</v>
+      </c>
+      <c r="G15" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2996.986084461212</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4142.241386413574</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E16" t="n">
+        <v>512</v>
+      </c>
+      <c r="F16" t="n">
+        <v>256</v>
+      </c>
+      <c r="G16" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3677.874319076538</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5257.66037607193</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E17" t="n">
+        <v>512</v>
+      </c>
+      <c r="F17" t="n">
+        <v>256</v>
+      </c>
+      <c r="G17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" t="n">
+        <v>6584.008889198303</v>
+      </c>
+      <c r="I17" t="n">
+        <v>9728.806594848633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>